<commit_message>
adding native mass spec
</commit_message>
<xml_diff>
--- a/kinetics/fit_michaelis-menten_parameters.xlsx
+++ b/kinetics/fit_michaelis-menten_parameters.xlsx
@@ -463,16 +463,16 @@
         <v>0.1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.06169441238611463</v>
+        <v>0.1557741599603557</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06961638598169714</v>
+        <v>1.320330699997939</v>
       </c>
       <c r="D2" t="n">
-        <v>8.655852317725843</v>
+        <v>720.0016475708619</v>
       </c>
       <c r="E2" t="n">
-        <v>46.80331780735393</v>
+        <v>8165.818992706494</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>0.25</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1785569254546778</v>
+        <v>0.1796149314902653</v>
       </c>
       <c r="C3" t="n">
-        <v>0.09096678140111472</v>
+        <v>0.09680101064877722</v>
       </c>
       <c r="D3" t="n">
-        <v>13.54221091348792</v>
+        <v>14.77303381886848</v>
       </c>
       <c r="E3" t="n">
-        <v>28.55890909187702</v>
+        <v>32.21023717138442</v>
       </c>
     </row>
     <row r="4">
@@ -497,16 +497,16 @@
         <v>0.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.2854472179242427</v>
+        <v>0.2819704518087692</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1040404405440425</v>
+        <v>0.1064695526243512</v>
       </c>
       <c r="D4" t="n">
-        <v>37.91028906677034</v>
+        <v>35.74680319584135</v>
       </c>
       <c r="E4" t="n">
-        <v>44.01148445999454</v>
+        <v>43.65975733495887</v>
       </c>
     </row>
     <row r="5">
@@ -514,16 +514,16 @@
         <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>0.4462144838943381</v>
+        <v>0.44820661939747</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1044017883459355</v>
+        <v>0.1020953591339012</v>
       </c>
       <c r="D5" t="n">
-        <v>56.48529894727904</v>
+        <v>56.26501872109692</v>
       </c>
       <c r="E5" t="n">
-        <v>37.76796972597</v>
+        <v>36.66750606300295</v>
       </c>
     </row>
     <row r="6">
@@ -531,16 +531,16 @@
         <v>2</v>
       </c>
       <c r="B6" t="n">
-        <v>1.023010415952592</v>
+        <v>0.9520651246702371</v>
       </c>
       <c r="C6" t="n">
-        <v>0.126629354706704</v>
+        <v>0.1257738226477255</v>
       </c>
       <c r="D6" t="n">
-        <v>91.35227489322216</v>
+        <v>83.82808101987764</v>
       </c>
       <c r="E6" t="n">
-        <v>28.03347271460406</v>
+        <v>28.18653246550533</v>
       </c>
     </row>
     <row r="7">
@@ -548,16 +548,16 @@
         <v>4</v>
       </c>
       <c r="B7" t="n">
-        <v>0.7474846544931081</v>
+        <v>0.6308632647241379</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1378509496422401</v>
+        <v>0.1071638995306426</v>
       </c>
       <c r="D7" t="n">
-        <v>75.27460106918234</v>
+        <v>62.99210369322052</v>
       </c>
       <c r="E7" t="n">
-        <v>36.49752055851479</v>
+        <v>29.64252898858475</v>
       </c>
     </row>
     <row r="8">
@@ -565,16 +565,16 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.6680898661772827</v>
+        <v>1.006159765946813</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1449981329052517</v>
+        <v>0.2101510814863432</v>
       </c>
       <c r="D8" t="n">
-        <v>92.74975829456318</v>
+        <v>234.8910139745124</v>
       </c>
       <c r="E8" t="n">
-        <v>47.88622933854307</v>
+        <v>89.82080068290801</v>
       </c>
     </row>
   </sheetData>
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -620,155 +620,172 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.03809171588904003</v>
+        <v>0.1557741599603557</v>
       </c>
       <c r="C2" t="n">
-        <v>0.03547810190742454</v>
+        <v>1.320330699997939</v>
       </c>
       <c r="D2" t="n">
-        <v>33.80273919164791</v>
+        <v>720.0016475708619</v>
       </c>
       <c r="E2" t="n">
-        <v>55.72590441620599</v>
+        <v>8165.818992706494</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="B3" t="n">
-        <v>0.07184288909711495</v>
+        <v>0.2993272919162709</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04696542689135814</v>
+        <v>18.41448525679804</v>
       </c>
       <c r="D3" t="n">
-        <v>9.987893533413802</v>
+        <v>1046.127254606185</v>
       </c>
       <c r="E3" t="n">
-        <v>27.5595505781932</v>
+        <v>68494.94296477536</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.1195875164132744</v>
+        <v>0.0667806581428067</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06437689000484174</v>
+        <v>0.04494289870527032</v>
       </c>
       <c r="D4" t="n">
-        <v>9.45261370114293</v>
+        <v>7.97067616542194</v>
       </c>
       <c r="E4" t="n">
-        <v>25.17735966528925</v>
+        <v>23.93440044715268</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>0.1186020960564543</v>
+        <v>0.1127038817917525</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0224471412243685</v>
+        <v>0.06406772903273765</v>
       </c>
       <c r="D5" t="n">
-        <v>81.80531731022947</v>
+        <v>8.100000418465058</v>
       </c>
       <c r="E5" t="n">
-        <v>39.70146776448353</v>
+        <v>23.55840123674946</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B6" t="n">
-        <v>0.0996461005319407</v>
+        <v>0.121973794398789</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01491073055178717</v>
+        <v>0.02191255739869373</v>
       </c>
       <c r="D6" t="n">
-        <v>48.59004806598271</v>
+        <v>83.62519403824095</v>
       </c>
       <c r="E6" t="n">
-        <v>21.66784190390853</v>
+        <v>38.265917453269</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B7" t="n">
-        <v>0.1076455097561416</v>
+        <v>0.1026354321943083</v>
       </c>
       <c r="C7" t="n">
-        <v>0.02337906607459791</v>
+        <v>0.01444862457844128</v>
       </c>
       <c r="D7" t="n">
-        <v>46.73111297108611</v>
+        <v>52.0089121669484</v>
       </c>
       <c r="E7" t="n">
-        <v>30.57112220501619</v>
+        <v>21.41370236851807</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.1392502551057721</v>
+        <v>0.1270491391543379</v>
       </c>
       <c r="C8" t="n">
-        <v>0.03681019606749091</v>
+        <v>0.01758759953094102</v>
       </c>
       <c r="D8" t="n">
-        <v>174.2339134833996</v>
+        <v>75.51309547453744</v>
       </c>
       <c r="E8" t="n">
-        <v>92.89016725103026</v>
+        <v>27.45721546977048</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B9" t="n">
-        <v>0.1286407001792204</v>
+        <v>0.1782536647860525</v>
       </c>
       <c r="C9" t="n">
-        <v>0.08804121619240081</v>
+        <v>0.06917189460336784</v>
       </c>
       <c r="D9" t="n">
-        <v>305.0936774624449</v>
+        <v>234.9463969776523</v>
       </c>
       <c r="E9" t="n">
-        <v>352.0893813641511</v>
+        <v>166.9064128778388</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3383682215738799</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.1663096831061791</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1205.983543701041</v>
+      </c>
+      <c r="E10" t="n">
+        <v>718.2568842891912</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>64</v>
       </c>
-      <c r="B10" t="n">
-        <v>0.09205150824375138</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.2695145345837223</v>
-      </c>
-      <c r="D10" t="n">
-        <v>553.8529832046801</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1814.985285987108</v>
+      <c r="B11" t="n">
+        <v>9.552327408485196</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2258.199396122136</v>
+      </c>
+      <c r="D11" t="n">
+        <v>69696.82615044792</v>
+      </c>
+      <c r="E11" t="n">
+        <v>16492763.8560122</v>
       </c>
     </row>
   </sheetData>
@@ -782,7 +799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -814,108 +831,125 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.006864968520578879</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>0.1557741599603557</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1.320330699997939</v>
       </c>
       <c r="D2" t="n">
-        <v>-81.65568004652816</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>720.0016475708619</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8165.818992706494</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="B3" t="n">
-        <v>0.2080881237526861</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.0632460880149277</v>
+        <v>0.1443705677821047</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>27.41608041080211</v>
-      </c>
-      <c r="E3" t="n">
-        <v>28.84665708263912</v>
+        <v>1389.234031426353</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.296073647534002</v>
+        <v>0.2049526988718987</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06109463598134737</v>
+        <v>0.06278461577733577</v>
       </c>
       <c r="D4" t="n">
-        <v>45.66397060086462</v>
+        <v>27.13314587072695</v>
       </c>
       <c r="E4" t="n">
-        <v>28.56221819377759</v>
+        <v>28.84813472897057</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>0.3473145122795658</v>
+        <v>0.2850997259707746</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0865686675918108</v>
+        <v>0.0623568594486017</v>
       </c>
       <c r="D5" t="n">
-        <v>69.57829519011287</v>
+        <v>42.12441135410582</v>
       </c>
       <c r="E5" t="n">
-        <v>46.6697312594351</v>
+        <v>28.53990016368526</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B6" t="n">
-        <v>0.4713513947787253</v>
+        <v>0.3312088497119743</v>
       </c>
       <c r="C6" t="n">
-        <v>0.2096425428305514</v>
+        <v>0.08795897663081605</v>
       </c>
       <c r="D6" t="n">
-        <v>145.8903567716825</v>
+        <v>62.96730488077809</v>
       </c>
       <c r="E6" t="n">
-        <v>138.6435415268439</v>
+        <v>46.32960041917794</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.3911881428211099</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.1540185436931057</v>
+      </c>
+      <c r="D7" t="n">
+        <v>107.5389382700949</v>
+      </c>
+      <c r="E7" t="n">
+        <v>99.75722055365519</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>8</v>
       </c>
-      <c r="B7" t="n">
-        <v>0.2988584913701983</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.03782999142990716</v>
-      </c>
-      <c r="D7" t="n">
-        <v>73.95495521430122</v>
-      </c>
-      <c r="E7" t="n">
-        <v>24.74207696014219</v>
+      <c r="B8" t="n">
+        <v>0.3087139360342603</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.07588263949559472</v>
+      </c>
+      <c r="D8" t="n">
+        <v>65.04785978094611</v>
+      </c>
+      <c r="E8" t="n">
+        <v>43.88316827577051</v>
       </c>
     </row>
   </sheetData>
@@ -964,16 +998,16 @@
         <v>0.1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0623527055040973</v>
+        <v>0.1557741599603557</v>
       </c>
       <c r="C2" t="n">
-        <v>0.03475842552325142</v>
+        <v>1.320330699997939</v>
       </c>
       <c r="D2" t="n">
-        <v>5.206399055221365</v>
+        <v>720.0016475708619</v>
       </c>
       <c r="E2" t="n">
-        <v>16.28352541423656</v>
+        <v>8165.818992706494</v>
       </c>
     </row>
     <row r="3">
@@ -981,16 +1015,16 @@
         <v>0.25</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1983607432498137</v>
+        <v>0.1972163559578891</v>
       </c>
       <c r="C3" t="n">
-        <v>0.08316000754957335</v>
+        <v>0.08387769871642223</v>
       </c>
       <c r="D3" t="n">
-        <v>8.926041553356345</v>
+        <v>9.116812901930063</v>
       </c>
       <c r="E3" t="n">
-        <v>17.41964403723877</v>
+        <v>17.93375182104504</v>
       </c>
     </row>
     <row r="4">
@@ -998,16 +1032,16 @@
         <v>0.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.3389104806336154</v>
+        <v>0.3322565953880512</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1427438343751831</v>
+        <v>0.140622714326631</v>
       </c>
       <c r="D4" t="n">
-        <v>25.79928251162977</v>
+        <v>24.94429461984245</v>
       </c>
       <c r="E4" t="n">
-        <v>38.19199320228873</v>
+        <v>37.4235498718166</v>
       </c>
     </row>
     <row r="5">
@@ -1015,16 +1049,16 @@
         <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>0.4110492915965743</v>
+        <v>0.4003183660118741</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1131707654390594</v>
+        <v>0.1122257417034107</v>
       </c>
       <c r="D5" t="n">
-        <v>37.45439549749413</v>
+        <v>35.27576275791493</v>
       </c>
       <c r="E5" t="n">
-        <v>32.95306529177601</v>
+        <v>32.0983405010467</v>
       </c>
     </row>
     <row r="6">
@@ -1032,16 +1066,16 @@
         <v>2</v>
       </c>
       <c r="B6" t="n">
-        <v>0.6397906257818574</v>
+        <v>0.6228080123652374</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1268879034651522</v>
+        <v>0.1313929088181478</v>
       </c>
       <c r="D6" t="n">
-        <v>76.70030811466727</v>
+        <v>76.59642675497331</v>
       </c>
       <c r="E6" t="n">
-        <v>39.7703633080007</v>
+        <v>42.26455184570866</v>
       </c>
     </row>
     <row r="7">
@@ -1049,16 +1083,16 @@
         <v>4</v>
       </c>
       <c r="B7" t="n">
-        <v>0.6071224836431662</v>
+        <v>0.6454639891955112</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1713661749583383</v>
+        <v>0.1203195561342442</v>
       </c>
       <c r="D7" t="n">
-        <v>71.0783843814385</v>
+        <v>85.84108957470642</v>
       </c>
       <c r="E7" t="n">
-        <v>53.65334868044145</v>
+        <v>40.43413544937631</v>
       </c>
     </row>
     <row r="8">
@@ -1066,16 +1100,16 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.9269407589265808</v>
+        <v>0.94549324815866</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2596184457370225</v>
+        <v>0.3308265982146518</v>
       </c>
       <c r="D8" t="n">
-        <v>210.655409704811</v>
+        <v>268.5386122059352</v>
       </c>
       <c r="E8" t="n">
-        <v>111.9854522587764</v>
+        <v>164.9667434820136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
lots of messing around, commit
</commit_message>
<xml_diff>
--- a/kinetics/fit_michaelis-menten_parameters.xlsx
+++ b/kinetics/fit_michaelis-menten_parameters.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,121 +460,87 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1557741599603557</v>
+        <v>0.2846463267861615</v>
       </c>
       <c r="C2" t="n">
-        <v>1.320330699997939</v>
+        <v>0.1043398433238548</v>
       </c>
       <c r="D2" t="n">
-        <v>720.0016475708619</v>
+        <v>36.58086042941272</v>
       </c>
       <c r="E2" t="n">
-        <v>8165.818992706494</v>
+        <v>43.1132574951154</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1796149314902653</v>
+        <v>0.445414301142183</v>
       </c>
       <c r="C3" t="n">
-        <v>0.09680101064877722</v>
+        <v>0.103740419815951</v>
       </c>
       <c r="D3" t="n">
-        <v>14.77303381886848</v>
+        <v>55.88985660735491</v>
       </c>
       <c r="E3" t="n">
-        <v>32.21023717138442</v>
+        <v>37.31226909245104</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0.2819704518087692</v>
+        <v>1.022202171787204</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1064695526243512</v>
+        <v>0.1252220349680019</v>
       </c>
       <c r="D4" t="n">
-        <v>35.74680319584135</v>
+        <v>91.13183221608833</v>
       </c>
       <c r="E4" t="n">
-        <v>43.65975733495887</v>
+        <v>27.69714476624361</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.44820661939747</v>
+        <v>0.7470045063311889</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1020953591339012</v>
+        <v>0.1373020961574731</v>
       </c>
       <c r="D5" t="n">
-        <v>56.26501872109692</v>
+        <v>75.10761254745285</v>
       </c>
       <c r="E5" t="n">
-        <v>36.66750606300295</v>
+        <v>36.31910062616479</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B6" t="n">
-        <v>0.9520651246702371</v>
+        <v>0.671653410744076</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1257738226477255</v>
+        <v>0.2168763703105202</v>
       </c>
       <c r="D6" t="n">
-        <v>83.82808101987764</v>
+        <v>104.3570997626826</v>
       </c>
       <c r="E6" t="n">
-        <v>28.18653246550533</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" t="n">
-        <v>0.6308632647241379</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.1071638995306426</v>
-      </c>
-      <c r="D7" t="n">
-        <v>62.99210369322052</v>
-      </c>
-      <c r="E7" t="n">
-        <v>29.64252898858475</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>8</v>
-      </c>
-      <c r="B8" t="n">
-        <v>1.006159765946813</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.2101510814863432</v>
-      </c>
-      <c r="D8" t="n">
-        <v>234.8910139745124</v>
-      </c>
-      <c r="E8" t="n">
-        <v>89.82080068290801</v>
+        <v>80.14709455730272</v>
       </c>
     </row>
   </sheetData>
@@ -588,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -620,172 +586,138 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1557741599603557</v>
+        <v>0.07066158777815634</v>
       </c>
       <c r="C2" t="n">
-        <v>1.320330699997939</v>
+        <v>0.0449838860631666</v>
       </c>
       <c r="D2" t="n">
-        <v>720.0016475708619</v>
+        <v>8.769461871849273</v>
       </c>
       <c r="E2" t="n">
-        <v>8165.818992706494</v>
+        <v>24.31678676628525</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.2993272919162709</v>
+        <v>0.1190545406875076</v>
       </c>
       <c r="C3" t="n">
-        <v>18.41448525679804</v>
+        <v>0.06338153880034189</v>
       </c>
       <c r="D3" t="n">
-        <v>1046.127254606185</v>
+        <v>8.967781545607851</v>
       </c>
       <c r="E3" t="n">
-        <v>68494.94296477536</v>
+        <v>23.88857758303758</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0667806581428067</v>
+        <v>0.1190396643177355</v>
       </c>
       <c r="C4" t="n">
-        <v>0.04494289870527032</v>
+        <v>0.02194461693610757</v>
       </c>
       <c r="D4" t="n">
-        <v>7.97067616542194</v>
+        <v>80.12324842923604</v>
       </c>
       <c r="E4" t="n">
-        <v>23.93440044715268</v>
+        <v>38.11268335067127</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.1127038817917525</v>
+        <v>0.1022871915939009</v>
       </c>
       <c r="C5" t="n">
-        <v>0.06406772903273765</v>
+        <v>0.01511340705421848</v>
       </c>
       <c r="D5" t="n">
-        <v>8.100000418465058</v>
+        <v>50.27995728452537</v>
       </c>
       <c r="E5" t="n">
-        <v>23.55840123674946</v>
+        <v>21.93256001587887</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B6" t="n">
-        <v>0.121973794398789</v>
+        <v>0.11601266129853</v>
       </c>
       <c r="C6" t="n">
-        <v>0.02191255739869373</v>
+        <v>0.02130724625608002</v>
       </c>
       <c r="D6" t="n">
-        <v>83.62519403824095</v>
+        <v>53.52731923887905</v>
       </c>
       <c r="E6" t="n">
-        <v>38.265917453269</v>
+        <v>28.52319458528442</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B7" t="n">
-        <v>0.1026354321943083</v>
+        <v>0.1434499211555939</v>
       </c>
       <c r="C7" t="n">
-        <v>0.01444862457844128</v>
+        <v>0.0400470315740712</v>
       </c>
       <c r="D7" t="n">
-        <v>52.0089121669484</v>
+        <v>174.3512973184723</v>
       </c>
       <c r="E7" t="n">
-        <v>21.41370236851807</v>
+        <v>98.14400082074457</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="B8" t="n">
-        <v>0.1270491391543379</v>
+        <v>0.1103844028159918</v>
       </c>
       <c r="C8" t="n">
-        <v>0.01758759953094102</v>
+        <v>0.07473510036095556</v>
       </c>
       <c r="D8" t="n">
-        <v>75.51309547453744</v>
+        <v>299.5321405639298</v>
       </c>
       <c r="E8" t="n">
-        <v>27.45721546977048</v>
+        <v>343.9001278329087</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="B9" t="n">
-        <v>0.1782536647860525</v>
+        <v>0.08128375133318556</v>
       </c>
       <c r="C9" t="n">
-        <v>0.06917189460336784</v>
+        <v>0.03838793937429889</v>
       </c>
       <c r="D9" t="n">
-        <v>234.9463969776523</v>
+        <v>531.1178558843972</v>
       </c>
       <c r="E9" t="n">
-        <v>166.9064128778388</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>32</v>
-      </c>
-      <c r="B10" t="n">
-        <v>0.3383682215738799</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.1663096831061791</v>
-      </c>
-      <c r="D10" t="n">
-        <v>1205.983543701041</v>
-      </c>
-      <c r="E10" t="n">
-        <v>718.2568842891912</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>64</v>
-      </c>
-      <c r="B11" t="n">
-        <v>9.552327408485196</v>
-      </c>
-      <c r="C11" t="n">
-        <v>2258.199396122136</v>
-      </c>
-      <c r="D11" t="n">
-        <v>69696.82615044792</v>
-      </c>
-      <c r="E11" t="n">
-        <v>16492763.8560122</v>
+        <v>361.1406948727565</v>
       </c>
     </row>
   </sheetData>
@@ -799,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -831,125 +763,87 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1557741599603557</v>
+        <v>0.2089723838861918</v>
       </c>
       <c r="C2" t="n">
-        <v>1.320330699997939</v>
+        <v>0.06345458279550857</v>
       </c>
       <c r="D2" t="n">
-        <v>720.0016475708619</v>
+        <v>27.84722785090121</v>
       </c>
       <c r="E2" t="n">
-        <v>8165.818992706494</v>
+        <v>29.15611984614574</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1443705677821047</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>0.2952245067045134</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.05930260759279541</v>
       </c>
       <c r="D3" t="n">
-        <v>1389.234031426353</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>45.00682710918372</v>
+      </c>
+      <c r="E3" t="n">
+        <v>27.51079944007955</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0.2049526988718987</v>
+        <v>0.3467205898241152</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06278461577733577</v>
+        <v>0.08505042591542948</v>
       </c>
       <c r="D4" t="n">
-        <v>27.13314587072695</v>
+        <v>69.09260901444512</v>
       </c>
       <c r="E4" t="n">
-        <v>28.84813472897057</v>
+        <v>45.70422210742688</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2850997259707746</v>
+        <v>0.4620496840997195</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0623568594486017</v>
+        <v>0.1993621637323383</v>
       </c>
       <c r="D5" t="n">
-        <v>42.12441135410582</v>
+        <v>137.9306852481118</v>
       </c>
       <c r="E5" t="n">
-        <v>28.53990016368526</v>
+        <v>129.4922811796211</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B6" t="n">
-        <v>0.3312088497119743</v>
+        <v>0.3041791465565507</v>
       </c>
       <c r="C6" t="n">
-        <v>0.08795897663081605</v>
+        <v>0.04056577760054302</v>
       </c>
       <c r="D6" t="n">
-        <v>62.96730488077809</v>
+        <v>70.63547659246252</v>
       </c>
       <c r="E6" t="n">
-        <v>46.32960041917794</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" t="n">
-        <v>0.3911881428211099</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.1540185436931057</v>
-      </c>
-      <c r="D7" t="n">
-        <v>107.5389382700949</v>
-      </c>
-      <c r="E7" t="n">
-        <v>99.75722055365519</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>8</v>
-      </c>
-      <c r="B8" t="n">
-        <v>0.3087139360342603</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.07588263949559472</v>
-      </c>
-      <c r="D8" t="n">
-        <v>65.04785978094611</v>
-      </c>
-      <c r="E8" t="n">
-        <v>43.88316827577051</v>
+        <v>25.23819177032362</v>
       </c>
     </row>
   </sheetData>
@@ -963,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -995,121 +889,87 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1557741599603557</v>
+        <v>0.3371803818198761</v>
       </c>
       <c r="C2" t="n">
-        <v>1.320330699997939</v>
+        <v>0.1424270396341275</v>
       </c>
       <c r="D2" t="n">
-        <v>720.0016475708619</v>
+        <v>25.28236516315839</v>
       </c>
       <c r="E2" t="n">
-        <v>8165.818992706494</v>
+        <v>37.72893239659942</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1972163559578891</v>
+        <v>0.4101194506870621</v>
       </c>
       <c r="C3" t="n">
-        <v>0.08387769871642223</v>
+        <v>0.1122839337273375</v>
       </c>
       <c r="D3" t="n">
-        <v>9.116812901930063</v>
+        <v>36.8795314424063</v>
       </c>
       <c r="E3" t="n">
-        <v>17.93375182104504</v>
+        <v>32.39534313174078</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0.3322565953880512</v>
+        <v>0.6390014956278058</v>
       </c>
       <c r="C4" t="n">
-        <v>0.140622714326631</v>
+        <v>0.1261592679687824</v>
       </c>
       <c r="D4" t="n">
-        <v>24.94429461984245</v>
+        <v>76.40037627412531</v>
       </c>
       <c r="E4" t="n">
-        <v>37.4235498718166</v>
+        <v>39.48170362753832</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.4003183660118741</v>
+        <v>0.6103373832746547</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1122257417034107</v>
+        <v>0.1669564840893531</v>
       </c>
       <c r="D5" t="n">
-        <v>35.27576275791493</v>
+        <v>71.20697678984563</v>
       </c>
       <c r="E5" t="n">
-        <v>32.0983405010467</v>
+        <v>52.06285077664751</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B6" t="n">
-        <v>0.6228080123652374</v>
+        <v>0.9166811474823728</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1313929088181478</v>
+        <v>0.2383119780642649</v>
       </c>
       <c r="D6" t="n">
-        <v>76.59642675497331</v>
+        <v>205.5669171897232</v>
       </c>
       <c r="E6" t="n">
-        <v>42.26455184570866</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" t="n">
-        <v>0.6454639891955112</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.1203195561342442</v>
-      </c>
-      <c r="D7" t="n">
-        <v>85.84108957470642</v>
-      </c>
-      <c r="E7" t="n">
-        <v>40.43413544937631</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>8</v>
-      </c>
-      <c r="B8" t="n">
-        <v>0.94549324815866</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.3308265982146518</v>
-      </c>
-      <c r="D8" t="n">
-        <v>268.5386122059352</v>
-      </c>
-      <c r="E8" t="n">
-        <v>164.9667434820136</v>
+        <v>102.2460469817051</v>
       </c>
     </row>
   </sheetData>

</xml_diff>